<commit_message>
hice codigo de profoirmas para enviar fichas tecnicas y verificar cantidades
</commit_message>
<xml_diff>
--- a/productos_agotados.xlsx
+++ b/productos_agotados.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,6 +27,13 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="10"/>
+      <sz val="12"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -52,17 +59,20 @@
       <bottom style="thin"/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -425,12 +435,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="63" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="75" customWidth="1" min="2" max="2"/>
+    <col width="125" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -446,26 +456,499 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>agotados</t>
+          <t>link</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>PFI2000</t>
+          <t>06222</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>REJILLA FILTRO PARA VENTILADOR 150x172, DIM 210x210x31MM IP54</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>-9</v>
+          <t>GUARDAMOTOR 25-40A</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>https://electricasbogota.com/es/downloads/dl/file/id/1032/product/6595/Chint - NS2 - Esp - Datasheets.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>06214</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>GUARDAMOTOR 13-18A UL</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>https://electricasbogota.com/es/downloads/dl/file/id/1032/product/6592/Chint - NS2 - Esp - Datasheets.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>09680</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>BRK 3X63A 230/400V 6KA C IEC</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>https://electricasbogota.com/es/downloads/dl/file/id/1059/product/6872/Chint - NB1 - Datasheet.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>68200</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>PLC XD3 8 ENTRADAS / 8 SALIDAS 2TRANSISTOR 6 RELE, 90-240VAC</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>https://electricasbogota.com/es/downloads/dl/file/id/24/product/1175/Xinje_-_PLC_XD_-_Hardware_manual.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>68200</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>PLC XD3 8 ENTRADAS / 8 SALIDAS 2TRANSISTOR 6 RELE, 90-240VAC</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>https://electricasbogota.com/es/downloads/dl/file/id/25/product/1175/Xinje_-_PLC_XD_-_Expansion_module_manual.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>68200</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>PLC XD3 8 ENTRADAS / 8 SALIDAS 2TRANSISTOR 6 RELE, 90-240VAC</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>https://electricasbogota.com/es/downloads/dl/file/id/30/product/1175/Xinje_-_PLC_XD_-_Instruction_manual.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>68200</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>PLC XD3 8 ENTRADAS / 8 SALIDAS 2TRANSISTOR 6 RELE, 90-240VAC</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>https://electricasbogota.com/es/downloads/dl/file/id/2129/product/1175/Xinje -SerieXD- BROSCHURE.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>68200</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>PLC XD3 8 ENTRADAS / 8 SALIDAS 2TRANSISTOR 6 RELE, 90-240VAC</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>https://electricasbogota.com/es/downloads/dl/file/id/2137/product/1175/Xinje -SerieXD3- DATASHEET.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>68200</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>PLC XD3 8 ENTRADAS / 8 SALIDAS 2TRANSISTOR 6 RELE, 90-240VAC</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>https://electricasbogota.com/es/downloads/dl/file/id/3321/product/1175/Xinje - PLC XD - Positioning control manual.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>68272</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>EXPANSION LATERAL 2 ENTRADAS ANALOGAS 12 BITS, 2 SALIDAS 10 BITS, VOLTAJE</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>https://electricasbogota.com/es/downloads/dl/file/id/25/product/12878/Xinje_-_PLC_XD_-_Expansion_module_manual.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>68272</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>EXPANSION LATERAL 2 ENTRADAS ANALOGAS 12 BITS, 2 SALIDAS 10 BITS, VOLTAJE</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>https://electricasbogota.com/es/downloads/dl/file/id/2131/product/12878/Xinje -SerieXD- MODULO DE E&amp;S IZQUIERDO.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>68272</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>EXPANSION LATERAL 2 ENTRADAS ANALOGAS 12 BITS, 2 SALIDAS 10 BITS, VOLTAJE</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>https://electricasbogota.com/es/downloads/dl/file/id/2133/product/12878/Xinje -SerieXD- MODULO DE ENTRADAS IZQUIERDO.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>68272</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>EXPANSION LATERAL 2 ENTRADAS ANALOGAS 12 BITS, 2 SALIDAS 10 BITS, VOLTAJE</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>https://electricasbogota.com/es/downloads/dl/file/id/2136/product/12878/Xinje -SerieXD- MODULO DE SALIDAS IZQUIERDO.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>68272</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>EXPANSION LATERAL 2 ENTRADAS ANALOGAS 12 BITS, 2 SALIDAS 10 BITS, VOLTAJE</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>https://electricasbogota.com/es/downloads/dl/file/id/3009/product/12878/Xinje_-_XD-2AD2DA-V-ED_-_Fast_Manual.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>67860</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>PANTALLA HMI TS2 4.3", 1 RS232, 1RS485 800*480 PIXELES ALIMENTACIÓN 24VDC</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>https://electricasbogota.com/es/downloads/dl/file/id/3107/product/14508/Xinje_-_HMI_TS2-TS3-TS5_-_Hardware_manual.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>67860</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>PANTALLA HMI TS2 4.3", 1 RS232, 1RS485 800*480 PIXELES ALIMENTACIÓN 24VDC</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>https://electricasbogota.com/es/downloads/dl/file/id/3310/product/14508/Xinje_-_TouchWin_Pro_-_Manual.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>67860</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>PANTALLA HMI TS2 4.3", 1 RS232, 1RS485 800*480 PIXELES ALIMENTACIÓN 24VDC</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>https://electricasbogota.com/es/downloads/dl/file/id/3315/product/14508/Xinje_-_HMI_TS_-_Communication_manual.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>68142</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>INTERFASE PLC XC - PC / PLC - HMI</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>https://electricasbogota.com/es/downloads/dl/file/id/32/product/1212/Xinje - XC - Manual.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>68142</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>INTERFASE PLC XC - PC / PLC - HMI</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>https://electricasbogota.com/es/downloads/dl/file/id/17/product/1212/Xinje -SerieXC-HARDWARE MANUAL.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>43026</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>FUENTE SW 24VDC/100W RIEL 90-264V</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>https://electricasbogota.com/es/downloads/dl/file/id/707/product/4011/EBCHQ - LP1100D - Ficha Técnica.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>09530</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>BREAKER 2X 3A, 10KA CURVA C, 230/400 VAC, IEC</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>https://electricasbogota.com/es/downloads/dl/file/id/1058/product/6779/Noark - EX9BH - Datasheets.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>09530</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>BREAKER 2X 3A, 10KA CURVA C, 230/400 VAC, IEC</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>https://electricasbogota.com/es/downloads/dl/file/id/2813/product/6779/noark_ex9bh_dataheet_ESP.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>53887</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>MONITOR DE VOLTAJE 3F 3 HILOS. VOLTAJE 175-345VAC. 1 RELE CONMUTABLE</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>https://electricasbogota.com/es/downloads/dl/file/id/3306/product/15144/Klemsan_-_Vigilantes_tensi_n_3F_P1D_-_Datasheet.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>1080063</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2153 BLOQUE DIST TRIP 3L 12 HUECOS 160A TAPAS LAT CON CUB</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>https://electricasbogota.com/es/downloads/dl/file/id/1421/product/9164/Onka - 2151_2153_2154 - Datasheets.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>1080063</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2153 BLOQUE DIST TRIP 3L 12 HUECOS 160A TAPAS LAT CON CUB</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>https://electricasbogota.com/es/downloads/dl/file/id/1428/product/9164/Onka_-_Bloques_de_distribuci_n_-_Datasheet.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>1080011</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2061 BLOQUE DIST 7 HUECOS 80A CON TAPA</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>https://electricasbogota.com/es/downloads/dl/file/id/1416/product/9147/Onka - 2061_2062_2064 - Datasheets.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>1080011</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2061 BLOQUE DIST 7 HUECOS 80A CON TAPA</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>https://electricasbogota.com/es/downloads/dl/file/id/1428/product/9147/Onka_-_Bloques_de_distribuci_n_-_Datasheet.pdf</t>
+        </is>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId27"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>